<commit_message>
Cite corrected workbook; add CV and registry lottery-hold options
Replace the workbook copy with the corrected version (Size Verification
nested payload-key layer, RFC 7685 rationale, clock model, Level 3
Results tab). RESULTS.md and README.md now cite the corrected values.
Adds cv_hold / reg_hold config options, a sequencing-only attack path
and hardening sweep jobs, plus tests that the measured sizes match the
corrected workbook and that the attacker's sequencing model matches the
simulator under each hold.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TXJ7s8Q6PbdYqCeuNUfpZe
</commit_message>
<xml_diff>
--- a/GPAExperiment/Birthmark_Traffic_Analysis_Catalog.xlsx
+++ b/GPAExperiment/Birthmark_Traffic_Analysis_Catalog.xlsx
@@ -12,6 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Simulation Parameters" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Size Verification" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Level 3 Experiment Design" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Level 3 Results" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -170,7 +171,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="30">
+  <cellXfs count="33">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
@@ -235,6 +236,15 @@
     <xf numFmtId="0" fontId="4" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -600,7 +610,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A35"/>
+  <dimension ref="A1:A43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -812,6 +822,55 @@
       <c r="A35" s="10" t="inlineStr">
         <is>
           <t>Prefer named, established methods over bespoke ones wherever a choice exists — a named method is independently checkable by a reviewer rather than needing to be justified from scratch. Reflected throughout: Substrate's own transport encryption over inventing one, RFC 7685's established padding range, the Hungarian algorithm for matching, Tor/Shadow's measurement-calibrated traffic model.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="11" t="inlineStr">
+        <is>
+          <t>Level 3 Results tab</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="10" t="inlineStr">
+        <is>
+          <t>The actual sweep outcome, run by Claude Code against this spec: neither attack beat</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="10" t="inlineStr">
+        <is>
+          <t>1/L anywhere from L=4 to L=40, including two hypothetical bounds stronger than any</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="10" t="inlineStr">
+        <is>
+          <t>attack actually built. One real, sub-threshold, uncalibrated signal (the sequencing</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="10" t="inlineStr">
+        <is>
+          <t>attack) is called out rather than folded into the headline pass. Two real errors the</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="10" t="inlineStr">
+        <is>
+          <t>experiment surfaced in this workbook (Size Verification's missing encryption layer, a</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="10" t="inlineStr">
+        <is>
+          <t>backwards RFC 7685 citation) are corrected in place, not just noted here.</t>
         </is>
       </c>
     </row>
@@ -2100,7 +2159,7 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="150" customHeight="1">
+    <row r="3" ht="200" customHeight="1">
       <c r="A3" s="6" t="inlineStr">
         <is>
           <t>Padding / traffic-size classes</t>
@@ -2118,7 +2177,7 @@
       </c>
       <c r="D3" s="12" t="inlineStr">
         <is>
-          <t>411B (Birthmark Standard's own credential-packet total) is a valid floor: the largest computed leg (gatekeeper fan-out, ~289B with transit overhead) sits well under it. 420–460B sits just above that floor and inside the range two universal, unavoidable network operations already occupy: TLS 1.3 ClientHello (RFC 7685 pads specifically to 256–511B, up to 508B, to avoid middlebox bugs) and DNSSEC/EDNS0 DNS responses (bounded by DNS's classic 512B UDP limit per RFC 1035; real measurements show these commonly landing just below 500B). A random draw within the range, rather than one fixed value, avoids the constancy itself becoming a signature. Range sufficiency is tested empirically in the Level 3 sweep, not assumed from this design choice alone.</t>
+          <t>411B (Birthmark Standard's own credential-packet total) is a valid floor: the largest measured leg (gatekeeper fan-out, 289B, confirmed via Claude Code's real-crypto Level 3 implementation) sits well under it. 420–460B sits just above that floor. CORRECTED: RFC 7685 was originally cited as evidence that TLS 1.3 ClientHellos commonly land in 256–511B — this was backwards. RFC 7685's padding extension exists to push ClientHellos OUT of that historically middlebox-problematic range, not into it. Measured against 360 real ClientHellos (Claude Code's Level 3 experiment), zero landed in the 442–482B wire window. The only real cover in that window is generic TLS 1.3 application-data records, and only about 2.1% of those happen to match — a real but much weaker blend-in claim than originally stated. DNSSEC/EDNS0 DNS responses (bounded by DNS's classic 512B UDP limit per RFC 1035) were not tested against this correction and the original claim there stands unless re-examined. Despite the weaker blend-in story, the Level 3 sweep result does not depend on it: neither attack beat the 1/L baseline anywhere in the tested range, and the actual protective mechanism turned out to be the per-hop timing/clock design, not traffic blend-in. A random draw within the padding range, rather than one fixed value, still avoids the constancy itself becoming a signature, independent of this correction.</t>
         </is>
       </c>
       <c r="E3" s="7" t="inlineStr">
@@ -2192,7 +2251,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D36"/>
+  <dimension ref="A1:D40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -2238,7 +2297,7 @@
         <v>33</v>
       </c>
       <c r="D2" s="20" t="n">
-        <v>186</v>
+        <v>235</v>
       </c>
     </row>
     <row r="3">
@@ -2302,7 +2361,7 @@
       <c r="D7" s="21" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="22" t="n"/>
+      <c r="A8" s="21" t="n"/>
       <c r="B8" s="19" t="inlineStr">
         <is>
           <t>Transit-layer overhead (ephemeral key + tag)</t>
@@ -2311,143 +2370,137 @@
       <c r="C8" s="19" t="n">
         <v>49</v>
       </c>
-      <c r="D8" s="22" t="n"/>
+      <c r="D8" s="21" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="18" t="inlineStr">
+      <c r="A9" s="22" t="n"/>
+      <c r="B9" s="19" t="inlineStr">
+        <is>
+          <t>Nested payload-key encryption layer (missed in original build-up)</t>
+        </is>
+      </c>
+      <c r="C9" s="19" t="n">
+        <v>49</v>
+      </c>
+      <c r="D9" s="22" t="n"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="18" t="inlineStr">
         <is>
           <t>Cred-3</t>
         </is>
       </c>
-      <c r="B9" s="19" t="inlineStr">
+      <c r="B10" s="19" t="inlineStr">
         <is>
           <t>Encrypted token</t>
         </is>
       </c>
-      <c r="C9" s="19" t="n">
+      <c r="C10" s="19" t="n">
         <v>81</v>
       </c>
-      <c r="D9" s="20" t="n">
-        <v>170</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="21" t="n"/>
-      <c r="B10" s="19" t="inlineStr">
-        <is>
-          <t>Key reference</t>
-        </is>
-      </c>
-      <c r="C10" s="19" t="n">
-        <v>8</v>
-      </c>
-      <c r="D10" s="21" t="n"/>
+      <c r="D10" s="20" t="n">
+        <v>219</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="21" t="n"/>
       <c r="B11" s="19" t="inlineStr">
         <is>
+          <t>Key reference</t>
+        </is>
+      </c>
+      <c r="C11" s="19" t="n">
+        <v>8</v>
+      </c>
+      <c r="D11" s="21" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="21" t="n"/>
+      <c r="B12" s="19" t="inlineStr">
+        <is>
           <t>PacketHash</t>
         </is>
       </c>
-      <c r="C11" s="19" t="n">
+      <c r="C12" s="19" t="n">
         <v>32</v>
       </c>
-      <c r="D11" s="21" t="n"/>
-    </row>
-    <row r="12">
-      <c r="A12" s="22" t="n"/>
-      <c r="B12" s="19" t="inlineStr">
+      <c r="D12" s="21" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="21" t="n"/>
+      <c r="B13" s="19" t="inlineStr">
         <is>
           <t>Transit-layer overhead</t>
         </is>
       </c>
-      <c r="C12" s="19" t="n">
+      <c r="C13" s="19" t="n">
         <v>49</v>
       </c>
-      <c r="D12" s="22" t="n"/>
-    </row>
-    <row r="13">
-      <c r="A13" s="18" t="inlineStr">
+      <c r="D13" s="21" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="22" t="n"/>
+      <c r="B14" s="19" t="inlineStr">
+        <is>
+          <t>Nested payload-key encryption layer (missed in original build-up)</t>
+        </is>
+      </c>
+      <c r="C14" s="19" t="n">
+        <v>49</v>
+      </c>
+      <c r="D14" s="22" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="18" t="inlineStr">
         <is>
           <t>ContA/B-1 / -2</t>
         </is>
       </c>
-      <c r="B13" s="19" t="inlineStr">
+      <c r="B15" s="19" t="inlineStr">
         <is>
           <t>ContentHash</t>
         </is>
       </c>
-      <c r="C13" s="19" t="n">
+      <c r="C15" s="19" t="n">
         <v>32</v>
       </c>
-      <c r="D13" s="20" t="n">
-        <v>113</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="21" t="n"/>
-      <c r="B14" s="19" t="inlineStr">
+      <c r="D15" s="20" t="n">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="21" t="n"/>
+      <c r="B16" s="19" t="inlineStr">
         <is>
           <t>Nonce n</t>
         </is>
       </c>
-      <c r="C14" s="19" t="n">
+      <c r="C16" s="19" t="n">
         <v>16</v>
       </c>
-      <c r="D14" s="21" t="n"/>
-    </row>
-    <row r="15">
-      <c r="A15" s="21" t="n"/>
-      <c r="B15" s="19" t="inlineStr">
+      <c r="D16" s="21" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="21" t="n"/>
+      <c r="B17" s="19" t="inlineStr">
         <is>
           <t>routing_code</t>
         </is>
       </c>
-      <c r="C15" s="19" t="n">
+      <c r="C17" s="19" t="n">
         <v>16</v>
       </c>
-      <c r="D15" s="21" t="n"/>
-    </row>
-    <row r="16">
-      <c r="A16" s="22" t="n"/>
-      <c r="B16" s="19" t="inlineStr">
-        <is>
-          <t>Transit-layer overhead</t>
-        </is>
-      </c>
-      <c r="C16" s="19" t="n">
-        <v>49</v>
-      </c>
-      <c r="D16" s="22" t="n"/>
-    </row>
-    <row r="17">
-      <c r="A17" s="18" t="inlineStr">
-        <is>
-          <t>ContA/B-3</t>
-        </is>
-      </c>
-      <c r="B17" s="19" t="inlineStr">
-        <is>
-          <t>ContentHash</t>
-        </is>
-      </c>
-      <c r="C17" s="19" t="n">
-        <v>32</v>
-      </c>
-      <c r="D17" s="20" t="n">
-        <v>97</v>
-      </c>
+      <c r="D17" s="21" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="21" t="n"/>
       <c r="B18" s="19" t="inlineStr">
         <is>
-          <t>Nonce n</t>
+          <t>Transit-layer overhead</t>
         </is>
       </c>
       <c r="C18" s="19" t="n">
-        <v>16</v>
+        <v>49</v>
       </c>
       <c r="D18" s="21" t="n"/>
     </row>
@@ -2455,7 +2508,7 @@
       <c r="A19" s="22" t="n"/>
       <c r="B19" s="19" t="inlineStr">
         <is>
-          <t>Transit-layer overhead</t>
+          <t>Nested payload-key encryption layer (missed in original build-up)</t>
         </is>
       </c>
       <c r="C19" s="19" t="n">
@@ -2466,30 +2519,30 @@
     <row r="20">
       <c r="A20" s="18" t="inlineStr">
         <is>
-          <t>GK fan-out (each)</t>
+          <t>ContA/B-3</t>
         </is>
       </c>
       <c r="B20" s="19" t="inlineStr">
         <is>
-          <t>PacketHash</t>
+          <t>ContentHash</t>
         </is>
       </c>
       <c r="C20" s="19" t="n">
         <v>32</v>
       </c>
       <c r="D20" s="20" t="n">
-        <v>289</v>
+        <v>146</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="21" t="n"/>
       <c r="B21" s="19" t="inlineStr">
         <is>
-          <t>Enc_PacketHash ciphertext+tag</t>
+          <t>Nonce n</t>
         </is>
       </c>
       <c r="C21" s="19" t="n">
-        <v>48</v>
+        <v>16</v>
       </c>
       <c r="D21" s="21" t="n"/>
     </row>
@@ -2497,131 +2550,131 @@
       <c r="A22" s="21" t="n"/>
       <c r="B22" s="19" t="inlineStr">
         <is>
+          <t>Transit-layer overhead</t>
+        </is>
+      </c>
+      <c r="C22" s="19" t="n">
+        <v>49</v>
+      </c>
+      <c r="D22" s="21" t="n"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="22" t="n"/>
+      <c r="B23" s="19" t="inlineStr">
+        <is>
+          <t>Nested payload-key encryption layer (missed in original build-up)</t>
+        </is>
+      </c>
+      <c r="C23" s="19" t="n">
+        <v>49</v>
+      </c>
+      <c r="D23" s="22" t="n"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="18" t="inlineStr">
+        <is>
+          <t>GK fan-out (each)</t>
+        </is>
+      </c>
+      <c r="B24" s="19" t="inlineStr">
+        <is>
+          <t>PacketHash</t>
+        </is>
+      </c>
+      <c r="C24" s="19" t="n">
+        <v>32</v>
+      </c>
+      <c r="D24" s="20" t="n">
+        <v>289</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="21" t="n"/>
+      <c r="B25" s="19" t="inlineStr">
+        <is>
+          <t>Enc_PacketHash ciphertext+tag</t>
+        </is>
+      </c>
+      <c r="C25" s="19" t="n">
+        <v>48</v>
+      </c>
+      <c r="D25" s="21" t="n"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="21" t="n"/>
+      <c r="B26" s="19" t="inlineStr">
+        <is>
           <t>Validator signature</t>
         </is>
       </c>
-      <c r="C22" s="19" t="n">
+      <c r="C26" s="19" t="n">
         <v>64</v>
       </c>
-      <c r="D22" s="21" t="n"/>
-    </row>
-    <row r="23">
-      <c r="A23" s="21" t="n"/>
-      <c r="B23" s="19" t="inlineStr">
-        <is>
-          <t>BlindShare_key</t>
-        </is>
-      </c>
-      <c r="C23" s="19" t="n">
-        <v>32</v>
-      </c>
-      <c r="D23" s="21" t="n"/>
-    </row>
-    <row r="24">
-      <c r="A24" s="21" t="n"/>
-      <c r="B24" s="19" t="inlineStr">
-        <is>
-          <t>C-signature</t>
-        </is>
-      </c>
-      <c r="C24" s="19" t="n">
-        <v>64</v>
-      </c>
-      <c r="D24" s="21" t="n"/>
-    </row>
-    <row r="25">
-      <c r="A25" s="22" t="n"/>
-      <c r="B25" s="19" t="inlineStr">
-        <is>
-          <t>Transit-layer overhead</t>
-        </is>
-      </c>
-      <c r="C25" s="19" t="n">
-        <v>49</v>
-      </c>
-      <c r="D25" s="22" t="n"/>
-    </row>
-    <row r="26">
-      <c r="A26" s="18" t="inlineStr">
-        <is>
-          <t>CV-1</t>
-        </is>
-      </c>
-      <c r="B26" s="19" t="inlineStr">
-        <is>
-          <t>Forwarded encrypted token</t>
-        </is>
-      </c>
-      <c r="C26" s="19" t="n">
-        <v>81</v>
-      </c>
-      <c r="D26" s="20" t="n">
-        <v>178</v>
-      </c>
+      <c r="D26" s="21" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="21" t="n"/>
       <c r="B27" s="19" t="inlineStr">
         <is>
-          <t>PacketHash wrapped under BlindShare_key + tag</t>
+          <t>BlindShare_key</t>
         </is>
       </c>
       <c r="C27" s="19" t="n">
-        <v>48</v>
+        <v>32</v>
       </c>
       <c r="D27" s="21" t="n"/>
     </row>
     <row r="28">
-      <c r="A28" s="22" t="n"/>
+      <c r="A28" s="21" t="n"/>
       <c r="B28" s="19" t="inlineStr">
         <is>
+          <t>C-signature</t>
+        </is>
+      </c>
+      <c r="C28" s="19" t="n">
+        <v>64</v>
+      </c>
+      <c r="D28" s="21" t="n"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="22" t="n"/>
+      <c r="B29" s="19" t="inlineStr">
+        <is>
           <t>Transit-layer overhead</t>
         </is>
       </c>
-      <c r="C28" s="19" t="n">
+      <c r="C29" s="19" t="n">
         <v>49</v>
       </c>
-      <c r="D28" s="22" t="n"/>
-    </row>
-    <row r="29">
-      <c r="A29" s="18" t="inlineStr">
-        <is>
-          <t>CV-2</t>
-        </is>
-      </c>
-      <c r="B29" s="19" t="inlineStr">
-        <is>
-          <t>Decision flag</t>
-        </is>
-      </c>
-      <c r="C29" s="19" t="n">
-        <v>4</v>
-      </c>
-      <c r="D29" s="20" t="n">
-        <v>165</v>
-      </c>
+      <c r="D29" s="22" t="n"/>
     </row>
     <row r="30">
-      <c r="A30" s="21" t="n"/>
+      <c r="A30" s="18" t="inlineStr">
+        <is>
+          <t>CV-1</t>
+        </is>
+      </c>
       <c r="B30" s="19" t="inlineStr">
         <is>
-          <t>Wrapped value (returned)</t>
+          <t>Forwarded encrypted token</t>
         </is>
       </c>
       <c r="C30" s="19" t="n">
-        <v>48</v>
-      </c>
-      <c r="D30" s="21" t="n"/>
+        <v>81</v>
+      </c>
+      <c r="D30" s="20" t="n">
+        <v>178</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="21" t="n"/>
       <c r="B31" s="19" t="inlineStr">
         <is>
-          <t>Validator signature</t>
+          <t>PacketHash wrapped under BlindShare_key + tag</t>
         </is>
       </c>
       <c r="C31" s="19" t="n">
-        <v>64</v>
+        <v>48</v>
       </c>
       <c r="D31" s="21" t="n"/>
     </row>
@@ -2640,59 +2693,113 @@
     <row r="33">
       <c r="A33" s="18" t="inlineStr">
         <is>
+          <t>CV-2</t>
+        </is>
+      </c>
+      <c r="B33" s="19" t="inlineStr">
+        <is>
+          <t>Decision flag</t>
+        </is>
+      </c>
+      <c r="C33" s="19" t="n">
+        <v>4</v>
+      </c>
+      <c r="D33" s="20" t="n">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="21" t="n"/>
+      <c r="B34" s="19" t="inlineStr">
+        <is>
+          <t>Wrapped value (returned)</t>
+        </is>
+      </c>
+      <c r="C34" s="19" t="n">
+        <v>48</v>
+      </c>
+      <c r="D34" s="21" t="n"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="21" t="n"/>
+      <c r="B35" s="19" t="inlineStr">
+        <is>
+          <t>Validator signature</t>
+        </is>
+      </c>
+      <c r="C35" s="19" t="n">
+        <v>64</v>
+      </c>
+      <c r="D35" s="21" t="n"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="22" t="n"/>
+      <c r="B36" s="19" t="inlineStr">
+        <is>
+          <t>Transit-layer overhead</t>
+        </is>
+      </c>
+      <c r="C36" s="19" t="n">
+        <v>49</v>
+      </c>
+      <c r="D36" s="22" t="n"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="18" t="inlineStr">
+        <is>
           <t>Reg-1 / Reg-2</t>
         </is>
       </c>
-      <c r="B33" s="19" t="inlineStr">
+      <c r="B37" s="19" t="inlineStr">
         <is>
           <t>ContentHash</t>
         </is>
       </c>
-      <c r="C33" s="19" t="n">
+      <c r="C37" s="19" t="n">
         <v>32</v>
       </c>
-      <c r="D33" s="20" t="n">
+      <c r="D37" s="20" t="n">
         <v>96</v>
       </c>
     </row>
-    <row r="34">
-      <c r="A34" s="22" t="n"/>
-      <c r="B34" s="19" t="inlineStr">
+    <row r="38">
+      <c r="A38" s="22" t="n"/>
+      <c r="B38" s="19" t="inlineStr">
         <is>
           <t>Server signature</t>
         </is>
       </c>
-      <c r="C34" s="19" t="n">
+      <c r="C38" s="19" t="n">
         <v>64</v>
       </c>
-      <c r="D34" s="22" t="n"/>
-    </row>
-    <row r="36" ht="45" customHeight="1">
-      <c r="A36" s="23" t="inlineStr">
-        <is>
-          <t>Every leg's raw size sits comfortably under 420 (the padding range floor), confirming padding up to the target range is possible for every leg without needing to pad down (impossible) or exceed the range (which would break the uniform-distribution guarantee). Re-run this if any component-size assumption changes (a different ECIES library's overhead, a different routing_code encoding, etc.).</t>
+      <c r="D38" s="22" t="n"/>
+    </row>
+    <row r="40" ht="75" customHeight="1">
+      <c r="A40" s="23" t="inlineStr">
+        <is>
+          <t>CORRECTED (via Claude Code's Level 3 implementation, which used real measured crypto rather than estimated component sizes): the original build-up omitted a nested payload-key encryption layer (+49B) on every relay leg (Cred-1/2/3, ContA/B-1/2/3) — real measured relay-leg sizes are 146–235B, not the original 97–186B estimate. GK fan-out (unaffected by this fix) remains the largest single leg at 289B, still comfortably under the 420B padding floor, so the padding target itself does not change — only this tab's arithmetic did. Re-run this if any component-size assumption changes (a different ECIES library's overhead, a different routing_code encoding, etc.).</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="17">
-    <mergeCell ref="A13:A16"/>
-    <mergeCell ref="D33:D34"/>
-    <mergeCell ref="D9:D12"/>
-    <mergeCell ref="D13:D16"/>
-    <mergeCell ref="A9:A12"/>
-    <mergeCell ref="A26:A28"/>
-    <mergeCell ref="A17:A19"/>
-    <mergeCell ref="D26:D28"/>
-    <mergeCell ref="A33:A34"/>
-    <mergeCell ref="A20:A25"/>
-    <mergeCell ref="A2:A8"/>
-    <mergeCell ref="D17:D19"/>
-    <mergeCell ref="D20:D25"/>
-    <mergeCell ref="D2:D8"/>
-    <mergeCell ref="D29:D32"/>
-    <mergeCell ref="A29:A32"/>
-    <mergeCell ref="A36:D36"/>
+    <mergeCell ref="A30:A32"/>
+    <mergeCell ref="A40:D40"/>
+    <mergeCell ref="D24:D29"/>
+    <mergeCell ref="D30:D32"/>
+    <mergeCell ref="A2:A9"/>
+    <mergeCell ref="A15:A19"/>
+    <mergeCell ref="D20:D23"/>
+    <mergeCell ref="A10:A14"/>
+    <mergeCell ref="A20:A23"/>
+    <mergeCell ref="A24:A29"/>
+    <mergeCell ref="D37:D38"/>
+    <mergeCell ref="A37:A38"/>
+    <mergeCell ref="D2:D9"/>
+    <mergeCell ref="A33:A36"/>
+    <mergeCell ref="D15:D19"/>
+    <mergeCell ref="D33:D36"/>
+    <mergeCell ref="D10:D14"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2704,7 +2811,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C31"/>
+  <dimension ref="A1:C34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -2729,7 +2836,7 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="90" customHeight="1">
+    <row r="2" ht="320" customHeight="1">
       <c r="A2" s="24" t="inlineStr">
         <is>
           <t>Simulation environment</t>
@@ -2737,7 +2844,7 @@
       </c>
       <c r="B2" s="7" t="inlineStr">
         <is>
-          <t>Custom-built, hosted in the same repo as the ProVerif models. Runs genuine TLS traffic for the padding blend-in component, plus a deliberately non-blending traffic type: large bulk transfers (unpadded, well outside the 256–511 byte window) and very small keepalive-style packets.</t>
+          <t>Custom-built, hosted in the same repo as the ProVerif models. Runs genuine TLS traffic for the padding blend-in component, plus a deliberately non-blending traffic type: large bulk transfers (unpadded, well outside the 256–511 byte window) and very small keepalive-style packets. Timing runs in virtual time, not real wall-clock time (necessary at sweep scale -- 15 settings x 200 runs). Byte sizes and record structure come from real TLS 1.3 output (actual ClientHellos and application-data records wrapping padded Birthmark payloads, generated offline via Python's ssl module) and byte-exact EDNS0/DNSSEC responses built offline, sampled from these measured pools during the simulation rather than opening a live connection per simulated packet. The pools must be internally diverse (multiple distinct real captures, not one sample repeated) -- a single fixed sample would reintroduce a constancy signal at the record-structure level even with the outer padded size randomized. The main sweep's observer reads the plaintext TLS record content-type byte and distinguishes UDP/53 (DNS) by port -- a real on-path observer can do this without decrypting anything, so not doing so under-powers the attack. Under this reading, ClientHello (0x16) and DNS traffic provide no cover regardless of size match; only other real TLS 1.3 application-data records (0x17) landing in the same wire-visible size range still blend in. The blend-in analysis separately reports survival with record type ignored, so the gap between the two readings is itself a reported Level 2 finding.</t>
         </is>
       </c>
       <c r="C2" s="7" t="inlineStr">
@@ -2746,7 +2853,7 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="90" customHeight="1">
+    <row r="3" ht="200" customHeight="1">
       <c r="A3" s="24" t="inlineStr">
         <is>
           <t>Background traffic</t>
@@ -2754,16 +2861,16 @@
       </c>
       <c r="B3" s="7" t="inlineStr">
         <is>
-          <t>Adapted from the Tor/Shadow 90/10 casual-vs-bulk client model (~90% transact then pause 1–60s uniformly at random, ~10% transact continuously). Content reuses the same real TLS/DNS traffic generation as the padding blend-in component, driven by this arrival pattern rather than a separate generator.</t>
+          <t>Adapted from the Tor/Shadow 90/10 casual-vs-bulk client model (~90% transact then pause 1–60s uniformly at random, ~10% transact continuously). Content reuses the same real TLS/DNS traffic generation as the padding blend-in component, driven by this arrival pattern rather than a separate generator. Volume: 25 background clients per node (500 total) for the main device-count sweep, held fixed across it. A separate sensitivity check varies background volume alone (0, 5, 25, 100 per node) at one mid-sweep device-count setting.</t>
         </is>
       </c>
       <c r="C3" s="7" t="inlineStr">
         <is>
-          <t>The ratio and pause-then-repeat structure transfer from the measurement-calibrated Tor/Shadow studies; Tor's KB-scale file sizes don't, since Birthmark's transactions are small and fixed-size.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="90" customHeight="1">
+          <t>The ratio and pause-then-repeat structure transfer from the measurement-calibrated Tor/Shadow studies; Tor's KB-scale file sizes don't, since Birthmark's transactions are small and fixed-size. Held fixed (rather than scaled with device count) specifically to avoid confounding the device-count sweep: if background volume changed alongside device count, a change in attack success couldn't be attributed to anonymity-set size versus blend-in quality.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="340" customHeight="1">
       <c r="A4" s="24" t="inlineStr">
         <is>
           <t>Correlation attack algorithm</t>
@@ -2771,315 +2878,552 @@
       </c>
       <c r="B4" s="7" t="inlineStr">
         <is>
-          <t>Jitter composes per hop, independently, via a "chance of transit" lottery: 10-second ticks, 8.33% release probability per tick, forced release at 30 ticks (5 min cap). Total delay to any point is the sum of one independent draw per hop traversed — a convolution with no clean closed form, computed empirically by Monte Carlo simulating the lottery process itself rather than deriving exact math. Matching is two-way: pool ContA and ContB terminal arrivals into one candidate set and match credential-chains against the pool via bipartite matching (Hungarian algorithm). Success means landing on either the true ContA or true ContB candidate.</t>
+          <t>Two stages — the observer is never told which arrivals are terminal or which channel they belong to; on the wire every packet is a generically-sized, generically-timed event, indistinguishable from a relay hop, a terminal arrival, or background traffic. (1) Chain reconstruction: at every node, correlate in/out events (an OUT event is a plausible relay of an IN event if their timing gap is consistent with one lottery draw), chaining these across hops to produce candidate end-to-end paths. Jitter composes per hop, independently, via a "chance of transit" lottery: 10-second ticks, 8.33% release probability per tick, forced release at 30 ticks (5 min cap). The true delay distribution is a convolution with no closed form; scored empirically via Monte Carlo simulation of the lottery process. (2) Cross-channel grouping: cluster candidate chains by common origin time, not by any type label, using the same likelihood scoring — resolved via bipartite matching (Hungarian algorithm). Success means correctly grouping the true credential-chain with either its true ContA or true ContB chain, never having labeled either by type in advance. Lottery clock model: each node runs one shared 10-second clock with a random phase offset; every held packet at that node rolls on the node's shared ticks, not its own arrival-based timer. A per-packet timer (starting fresh at arrival) would preserve the device's original transmission phase exactly through every hop -- verified: arrival phase and terminal-hop phase are identical to machine precision under that model, regardless of how many ticks elapsed -- letting an observer match packets by sub-tick phase alone, a leak severe enough to dominate the results. The main sweep runs under the shared node-clock model; one small additional run under the per-packet-timer model quantifies how large that leak would have been, reported separately as a demonstration of why the shared-clock model is necessary, not just preferred. The device itself holds one packet per channel before each first hop, under the same lottery mechanism -- verified: a single shared device-wide clock puts all three first-hop departures on the same phase, letting Stage 2 cluster them even with device IP hidden, the same leak as the node-clock issue, moved to the device. Fix: each channel's hold at the device uses its own independently, freshly drawn random phase -- NOT a fixed phase assigned per channel type shared across devices, which would leak channel type through phase and undo the type-agnostic Stage 2 grouping. One small probe run under a single shared device clock quantifies the leak this avoids.</t>
         </is>
       </c>
       <c r="C4" s="7" t="inlineStr">
         <is>
-          <t>Independent per-hop draws increase total timing uncertainty for the attacker versus a single end-to-end draw, since independent variances add. The adversary only needs one content channel, not both, since either carries the full ContentHash. Baseline stays exactly 1/L under pooled matching (2 correct targets in a 2L-sized pool cancels to 1/L, same as unpooled).</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="90" customHeight="1">
+          <t>An oracle that hands the attacker terminal-arrival and channel-type labels tests only whether labeled candidates can be correlated — a much weaker question than whether the attacker can find which packets matter at all, which is what a real passive observer actually faces and what Semantic Non-Assembly needs to survive. Node role sharing across channels means even full topology knowledge doesn't legitimately grant terminal-arrival identity. Stage 1 also serves as the non-blending-traffic sanity check without a separate classifier: bulk/keepalive traffic won't produce a jitter-consistent in/out pattern, so it's filtered naturally. Independent per-hop draws increase total timing uncertainty for the attacker versus a single end-to-end draw, since independent variances add. Baseline stays exactly 1/L under pooled matching (2 correct targets in a 2L-sized pool cancels to 1/L).</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="150" customHeight="1">
       <c r="A5" s="24" t="inlineStr">
         <is>
-          <t>Success criterion</t>
+          <t>Origin-anchored trace (separate report)</t>
         </is>
       </c>
       <c r="B5" s="7" t="inlineStr">
         <is>
-          <t>Two-part: (1) raw pairing accuracy vs. the 1/L chance baseline; (2) calibration — among predictions made with high confidence (the score gap between top and runner-up candidates), what fraction are actually correct.</t>
+          <t>Additional attack, reported separately from the specified attack, not folded into its results: score the device's observed first-hop departure (Device→A/D/G, which carries the device's real IP if no IP-hiding layer sits in front of it) directly against content-terminal arrivals — only 2 relay draws of accumulated jitter rather than a full chain reconstruction on both sides, since the departure time is directly observed, not inferred.</t>
         </is>
       </c>
       <c r="C5" s="7" t="inlineStr">
         <is>
-          <t>An attacker can score above chance on accuracy while still failing calibration if it can't tell its correct guesses from its wrong ones — a materially weaker privacy failure than accuracy with good calibration.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="90" customHeight="1">
+          <t>Tests a different precondition than the rest of this experiment: whether the device's IP is hidden at all, which the paper requires ("no intermediary on either path ever observes the device's originating network address") but explicitly defers the mechanism for ("an anonymizing relay layer... is an implementation choice"). If no such layer is modeled, this attack succeeds near 100% — informative about why that layer is load-bearing, but a result about an unmodeled layer, not about Birthmark's timing/padding defenses. Reporting it folded into the main results would misattribute the failure. OPEN: whether the simulator models a generic IP-hiding layer for the first hop, or leaves it out of scope with this result standing as the demonstration of why it's needed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="220" customHeight="1">
       <c r="A6" s="24" t="inlineStr">
         <is>
-          <t>Scale parameters</t>
+          <t>Quorum→registry sequencing</t>
         </is>
       </c>
       <c r="B6" s="7" t="inlineStr">
         <is>
-          <t>20-node pool, fully connected, supplying all submission-server roles (relay, credential processor C, gatekeeper/match board). 4 validators, fixed across the sweep — devices split evenly across them at whatever count the current sweep run is using (e.g., 40 devices → 10 per validator, 200 devices → 50 per validator).</t>
+          <t>Additional attack, reported alongside the specified one: score GK fan-out timing against Reg-1/Reg-2 gossip timing. Requires a default for when F/I actually post: F/I poll the match boards on the same 10-second tick as the lottery mechanism and post as soon as they observe a 2-of-3 quorum. Experiment result: the sequencing signal traces to C→validator (CV-1/2) having no lottery hold at all — the round trip fires immediately, letting an observer detect credential-chain endings over 99% of the time and giving the sequencing attack its (sub-1/L but real, ~4–6x above true chance) signal. A lottery hold at CV-1/2, or at F/I before posting to the registry, is the concrete next hardening step to close even this weak residual signal — not required by the current result, since it stays under threshold, but a clean fix given the source is now identified.</t>
+        </is>
+      </c>
+      <c r="C6" s="7" t="inlineStr">
+        <is>
+          <t>Entirely within already-confirmed scope (GK-1/2/3 and Reg-1/2 are both already in the GPA's vantage point) — tests whether the protocol's own observable sequencing leaks a correlation the specified attack doesn't capture, not an unrelated layer. The polling default reuses an existing time granularity rather than inventing a new one; flagged as an assumption, not a confirmed design decision.</t>
         </is>
       </c>
     </row>
     <row r="7" ht="90" customHeight="1">
       <c r="A7" s="24" t="inlineStr">
         <is>
-          <t>Submission rate / sweep methodology</t>
+          <t>Success criterion</t>
         </is>
       </c>
       <c r="B7" s="7" t="inlineStr">
         <is>
-          <t>Sweep across roughly L=5 to L=25 (Little's Law: L = devices ÷ mean interval × mean jitter; table below) rather than committing to one device count, 200 independent runs per L value. The lowest L at which the attack still succeeds becomes the floor real traffic must maintain; synthetic traffic tops up volume only below that floor, targeted at whichever specific leg-pairings the attack actually exploits rather than padded uniformly everywhere.</t>
+          <t>Two-part: (1) raw pairing accuracy vs. the 1/L chance baseline; (2) calibration — among predictions made with high confidence (the score gap between top and runner-up candidates), what fraction are actually correct.</t>
         </is>
       </c>
       <c r="C7" s="7" t="inlineStr">
         <is>
-          <t>Turns "is 40 enough?" into a measured scaling curve instead of a single arbitrary number, and makes any dummy-traffic use a targeted response to a measured threshold rather than volume for its own sake.</t>
+          <t>An attacker can score above chance on accuracy while still failing calibration if it can't tell its correct guesses from its wrong ones — a materially weaker privacy failure than accuracy with good calibration.</t>
         </is>
       </c>
     </row>
     <row r="8" ht="90" customHeight="1">
       <c r="A8" s="24" t="inlineStr">
         <is>
-          <t>GPA tap scope</t>
+          <t>Scale parameters</t>
         </is>
       </c>
       <c r="B8" s="7" t="inlineStr">
         <is>
-          <t>Global passive observer: sees public relay hops (Cred/ContA/ContB), C↔validator (CV-1/2), C→gatekeeper fan-out (GK-1/2/3), and the final registry postings (Reg-1/2). Does not see gatekeeper-to-match-board (Post-1/2/3) or the internal F/I-to-entry-node step. Has compromised no nodes.</t>
-        </is>
-      </c>
-      <c r="C8" s="7" t="inlineStr">
-        <is>
-          <t>Fall back to an imperfect observer if this proves too strong to get a meaningful result against.</t>
+          <t>20-node pool, fully connected, supplying all submission-server roles (relay, credential processor C, gatekeeper/match board). 4 validators, fixed across the sweep — devices split evenly across them at whatever count the current sweep run is using (e.g., 40 devices → 10 per validator, 200 devices → 50 per validator).</t>
         </is>
       </c>
     </row>
     <row r="9" ht="90" customHeight="1">
       <c r="A9" s="24" t="inlineStr">
         <is>
+          <t>Submission rate / sweep methodology</t>
+        </is>
+      </c>
+      <c r="B9" s="7" t="inlineStr">
+        <is>
+          <t>Sweep across roughly L=5 to L=25 (Little's Law: L = devices ÷ mean interval × mean jitter; table below) rather than committing to one device count, 200 independent runs per L value. The lowest L at which the attack still succeeds becomes the floor real traffic must maintain; synthetic traffic tops up volume only below that floor, targeted at whichever specific leg-pairings the attack actually exploits rather than padded uniformly everywhere.</t>
+        </is>
+      </c>
+      <c r="C9" s="7" t="inlineStr">
+        <is>
+          <t>Turns "is 40 enough?" into a measured scaling curve instead of a single arbitrary number, and makes any dummy-traffic use a targeted response to a measured threshold rather than volume for its own sake.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="150" customHeight="1">
+      <c r="A10" s="24" t="inlineStr">
+        <is>
+          <t>Ingress anonymity (devices vs. background)</t>
+        </is>
+      </c>
+      <c r="B10" s="7" t="inlineStr">
+        <is>
+          <t>Every external→node event, from devices and background clients alike, is observed identically as "external → node X" with no source identity in the main attack. Stage 2 works from Stage 1's output alone. Only the separate origin-anchored section sees device IPs.</t>
+        </is>
+      </c>
+      <c r="C10" s="7" t="inlineStr">
+        <is>
+          <t>Necessary for the origin-anchored trace's separation to actually hold: if background senders kept visible IPs while device IPs were hidden, the mere absence of a visible IP would itself distinguish devices from background traffic, independent of anything about size or timing -- the same category of leak as the record-type and device-clock issues above.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="24" t="inlineStr">
+        <is>
+          <t>GPA tap scope</t>
+        </is>
+      </c>
+      <c r="B11" s="7" t="inlineStr">
+        <is>
+          <t>Global passive observer: sees public relay hops (Cred/ContA/ContB), C↔validator (CV-1/2), C→gatekeeper fan-out (GK-1/2/3), and the final registry postings (Reg-1/2). Does not see gatekeeper-to-match-board (Post-1/2/3) or the internal F/I-to-entry-node step. Has compromised no nodes.</t>
+        </is>
+      </c>
+      <c r="C11" s="7" t="inlineStr">
+        <is>
+          <t>Fall back to an imperfect observer if this proves too strong to get a meaningful result against.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="150" customHeight="1">
+      <c r="A12" s="7" t="inlineStr">
+        <is>
           <t>Registry intake and gossip</t>
         </is>
       </c>
-      <c r="B9" s="7" t="inlineStr">
+      <c r="B12" s="7" t="inlineStr">
         <is>
           <t>F/I is co-located with a blockchain node in the same Registry node, so the submission-to-entry-node step is internal, not network-observable; only the subsequent gossip fan-out is external. Substrate's transport (libp2p + Noise) encrypts gossip content hop-to-hop by default, so signatures aren't plaintext to an outside GPA — though every node along the gossip path sees them decrypted. Size and timing metadata aren't covered by that encryption and remain in scope.</t>
         </is>
       </c>
-      <c r="C9" s="7" t="inlineStr">
+      <c r="C12" s="7" t="inlineStr">
         <is>
           <t>Stem/fluff (Dandelion++-style) gossip restructuring is the intended direction for protecting which node originated a submission, deferred to a later version — it defends against a node-level observer, a different adversary than this experiment's GPA.</t>
         </is>
       </c>
     </row>
-    <row r="10" ht="90" customHeight="1">
-      <c r="A10" s="24" t="inlineStr">
+    <row r="13" ht="220" customHeight="1">
+      <c r="A13" s="24" t="inlineStr">
         <is>
           <t>Tech stack</t>
         </is>
       </c>
-      <c r="B10" s="7" t="inlineStr">
-        <is>
-          <t>Python. scipy.optimize.linear_sum_assignment provides the Hungarian algorithm for bipartite matching; asyncio maps cleanly onto the per-hop lottery (each held packet as a task rolling its release probability each tick); ssl gives genuine TLS.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="28" t="inlineStr">
+      <c r="B13" s="7" t="inlineStr">
+        <is>
+          <t>Python. scipy.optimize.linear_sum_assignment provides the Hungarian algorithm for bipartite matching; ssl gives genuine TLS. Lottery timing, CLARIFIED to close an ambiguity Claude Code correctly flagged: "each held packet as a task rolling its release probability each tick" reads naturally as an independent per-packet timer, which is the LEAKY version — confirmed by experiment, it lets an observer pair packets by shared sub-tick phase, defeating both the relay-hop and device-side clock defenses at once. The correct implementation is one shared clock per role, not per packet: one shared, randomly-phased clock per relay node (every packet held at that node rolls on the same ticks, erasing individual arrival phase), and one independently, freshly-drawn phase per channel at the device (so the device's three simultaneous first-hop departures don't share a phase either). Implement the shared clock as its own recurring task that wakes each held packet's check, rather than giving each packet its own independent timer.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="28" t="inlineStr">
         <is>
           <t>Little's Law sweep: L = (devices / mean interval) × mean jitter (2 min)</t>
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="17" t="inlineStr">
+    <row r="16">
+      <c r="A16" s="17" t="inlineStr">
         <is>
           <t>Devices</t>
         </is>
       </c>
-      <c r="B13" s="17" t="inlineStr">
+      <c r="B16" s="17" t="inlineStr">
         <is>
           <t>Mean interval (min)</t>
         </is>
       </c>
-      <c r="C13" s="17" t="inlineStr">
+      <c r="C16" s="17" t="inlineStr">
         <is>
           <t>L (in-flight anonymity set)</t>
         </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="19" t="n">
-        <v>40</v>
-      </c>
-      <c r="B14" s="19" t="n">
-        <v>10</v>
-      </c>
-      <c r="C14" s="19" t="n">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="19" t="n">
-        <v>40</v>
-      </c>
-      <c r="B15" s="19" t="n">
-        <v>15</v>
-      </c>
-      <c r="C15" s="19" t="n">
-        <v>5.3</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="19" t="n">
-        <v>40</v>
-      </c>
-      <c r="B16" s="19" t="n">
-        <v>20</v>
-      </c>
-      <c r="C16" s="19" t="n">
-        <v>4</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="19" t="n">
-        <v>80</v>
+        <v>40</v>
       </c>
       <c r="B17" s="19" t="n">
         <v>10</v>
       </c>
       <c r="C17" s="19" t="n">
-        <v>16</v>
+        <v>8</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="19" t="n">
-        <v>80</v>
+        <v>40</v>
       </c>
       <c r="B18" s="19" t="n">
         <v>15</v>
       </c>
       <c r="C18" s="19" t="n">
-        <v>10.7</v>
+        <v>5.3</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="19" t="n">
-        <v>80</v>
+        <v>40</v>
       </c>
       <c r="B19" s="19" t="n">
         <v>20</v>
       </c>
       <c r="C19" s="19" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="19" t="n">
-        <v>120</v>
+        <v>80</v>
       </c>
       <c r="B20" s="19" t="n">
         <v>10</v>
       </c>
       <c r="C20" s="19" t="n">
-        <v>24</v>
+        <v>16</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="19" t="n">
-        <v>120</v>
+        <v>80</v>
       </c>
       <c r="B21" s="19" t="n">
         <v>15</v>
       </c>
       <c r="C21" s="19" t="n">
-        <v>16</v>
+        <v>10.7</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="19" t="n">
-        <v>120</v>
+        <v>80</v>
       </c>
       <c r="B22" s="19" t="n">
         <v>20</v>
       </c>
       <c r="C22" s="19" t="n">
-        <v>12</v>
+        <v>8</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="19" t="n">
-        <v>160</v>
+        <v>120</v>
       </c>
       <c r="B23" s="19" t="n">
         <v>10</v>
       </c>
       <c r="C23" s="19" t="n">
-        <v>32</v>
+        <v>24</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="19" t="n">
-        <v>160</v>
+        <v>120</v>
       </c>
       <c r="B24" s="19" t="n">
         <v>15</v>
       </c>
       <c r="C24" s="19" t="n">
-        <v>21.3</v>
+        <v>16</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="19" t="n">
-        <v>160</v>
+        <v>120</v>
       </c>
       <c r="B25" s="19" t="n">
         <v>20</v>
       </c>
       <c r="C25" s="19" t="n">
-        <v>16</v>
+        <v>12</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="19" t="n">
-        <v>200</v>
+        <v>160</v>
       </c>
       <c r="B26" s="19" t="n">
         <v>10</v>
       </c>
       <c r="C26" s="19" t="n">
-        <v>40</v>
+        <v>32</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="19" t="n">
-        <v>200</v>
+        <v>160</v>
       </c>
       <c r="B27" s="19" t="n">
         <v>15</v>
       </c>
       <c r="C27" s="19" t="n">
-        <v>26.7</v>
+        <v>21.3</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="19" t="n">
-        <v>200</v>
+        <v>160</v>
       </c>
       <c r="B28" s="19" t="n">
         <v>20</v>
       </c>
       <c r="C28" s="19" t="n">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="19" t="n">
+        <v>200</v>
+      </c>
+      <c r="B29" s="19" t="n">
+        <v>10</v>
+      </c>
+      <c r="C29" s="19" t="n">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="19" t="n">
+        <v>200</v>
+      </c>
+      <c r="B30" s="19" t="n">
+        <v>15</v>
+      </c>
+      <c r="C30" s="19" t="n">
+        <v>26.7</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="19" t="n">
+        <v>200</v>
+      </c>
+      <c r="B31" s="19" t="n">
         <v>20</v>
       </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="19" t="n"/>
-      <c r="B29" s="19" t="n"/>
-      <c r="C29" s="19" t="n"/>
-    </row>
-    <row r="30">
-      <c r="A30" s="19" t="n"/>
-      <c r="B30" s="19" t="n"/>
-      <c r="C30" s="19" t="n"/>
-    </row>
-    <row r="31">
-      <c r="A31" s="19" t="n"/>
-      <c r="B31" s="19" t="n"/>
-      <c r="C31" s="19" t="n"/>
+      <c r="C31" s="19" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="19" t="n"/>
+      <c r="B32" s="19" t="n"/>
+      <c r="C32" s="19" t="n"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="19" t="n"/>
+      <c r="B33" s="19" t="n"/>
+      <c r="C33" s="19" t="n"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="19" t="n"/>
+      <c r="B34" s="19" t="n"/>
+      <c r="C34" s="19" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A12:C12"/>
-  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C10"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="26" customWidth="1" min="1" max="1"/>
+    <col width="60" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="17" t="inlineStr">
+        <is>
+          <t>Finding</t>
+        </is>
+      </c>
+      <c r="B1" s="17" t="inlineStr">
+        <is>
+          <t>Result</t>
+        </is>
+      </c>
+      <c r="C1" s="17" t="inlineStr">
+        <is>
+          <t>Read</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="100" customHeight="1">
+      <c r="A2" s="24" t="inlineStr">
+        <is>
+          <t>Headline result</t>
+        </is>
+      </c>
+      <c r="B2" s="7" t="inlineStr">
+        <is>
+          <t>Neither the main attack nor the sequencing attack beat the 1/L chance baseline anywhere across the full sweep, L = 4 to L = 40 (200 runs per setting, 15 workbook settings).</t>
+        </is>
+      </c>
+      <c r="C2" s="30" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="100" customHeight="1">
+      <c r="A3" s="24" t="inlineStr">
+        <is>
+          <t>Ground-truth bounds</t>
+        </is>
+      </c>
+      <c r="B3" s="7" t="inlineStr">
+        <is>
+          <t>Even an attacker handed true terminal labels, or handed perfect chain reconstruction for free, still stays under 1/L at every setting. This isn't "the specific attack implementation was weak" — the timing signal available is insufficient even for a much stronger hypothetical attacker than the one that was actually built.</t>
+        </is>
+      </c>
+      <c r="C3" s="30" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="100" customHeight="1">
+      <c r="A4" s="24" t="inlineStr">
+        <is>
+          <t>Sanity check: lottery disabled</t>
+        </is>
+      </c>
+      <c r="B4" s="7" t="inlineStr">
+        <is>
+          <t>With the lottery mechanism turned off, the same attack code pairs 99.2% of submissions correctly — confirms the attack machinery itself works; the result above is the timing defense doing real work, not an incompetent adversary.</t>
+        </is>
+      </c>
+      <c r="C4" s="30" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="100" customHeight="1">
+      <c r="A5" s="24" t="inlineStr">
+        <is>
+          <t>Sequencing attack (validator reply → registry posts)</t>
+        </is>
+      </c>
+      <c r="B5" s="7" t="inlineStr">
+        <is>
+          <t>Stays under 1/L (~0.58/L), but true chance for this specific attack is ~5x lower than 1/L (the real pairing window is wider than the 2 minutes L is calibrated against), so this is a real, ~4–6x-above-chance signal, not zero signal. Calibration saves it: no prediction was ever confident, and top-decile accuracy is barely above overall accuracy — an attacker can't act on a signal it can't distinguish from noise. Traced to CV-1/2 (C→validator) having no lottery hold at all; see Level 3 Experiment Design, row 6, for the concrete fix.</t>
+        </is>
+      </c>
+      <c r="C5" s="31" t="inlineStr">
+        <is>
+          <t>WATCH</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="100" customHeight="1">
+      <c r="A6" s="24" t="inlineStr">
+        <is>
+          <t>Origin-anchored trace (separate report)</t>
+        </is>
+      </c>
+      <c r="B6" s="7" t="inlineStr">
+        <is>
+          <t>Device IP → content-terminal tracing, skipping the credential chain entirely, still fails under the correct clock model (0.05–0.11%), only succeeding (99.9%) when the per-packet-timer bug is reintroduced. Confirms the relay-node clock defense protects the credential↔content link even when device identity is already known — the deferred IP-hiding layer is still a real requirement on its own terms, but its absence would not by itself reopen this correlation.</t>
+        </is>
+      </c>
+      <c r="C6" s="30" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="100" customHeight="1">
+      <c r="A7" s="24" t="inlineStr">
+        <is>
+          <t>Clock-model ambiguity, resolved by measurement</t>
+        </is>
+      </c>
+      <c r="B7" s="7" t="inlineStr">
+        <is>
+          <t>The two clock leaks (per-packet relay timers, shared device clock), run together: 65.9% paired, 91% confident on the top decile. Each fix blocks one stage independently — node-wide relay clock blocks hop tracing (98% with the leaky version); per-channel device phase blocks origin grouping (68% with the leaky version, given true chains). Both are now written unambiguously into the Level 3 Experiment Design tab's Tech stack row.</t>
+        </is>
+      </c>
+      <c r="C7" s="30" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="100" customHeight="1">
+      <c r="A8" s="24" t="inlineStr">
+        <is>
+          <t>Workbook errors found by the experiment, now corrected</t>
+        </is>
+      </c>
+      <c r="B8" s="7" t="inlineStr">
+        <is>
+          <t>(1) Size Verification omitted a nested payload-key encryption layer (+49B) on every relay leg — real measured sizes are 146–235B, not 97–186B; GK fan-out remains the largest leg at 289B, so the padding target itself is unaffected, only the tab's arithmetic was wrong. (2) RFC 7685 was cited backwards in Simulation Parameters — it pads ClientHellos OUT of the 256–511B range, not into it; 0 of 360 real ClientHellos landed in the 442–482B window. Only generic TLS 1.3 app-data records provide real cover, at ~2.1%. Neither error affects the headline result, which turns out to rest on the timing/clock defense, not traffic blend-in.</t>
+        </is>
+      </c>
+      <c r="C8" s="31" t="inlineStr">
+        <is>
+          <t>CORRECTED</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="100" customHeight="1">
+      <c r="A9" s="24" t="inlineStr">
+        <is>
+          <t>Assumptions the results rest on</t>
+        </is>
+      </c>
+      <c r="B9" s="7" t="inlineStr">
+        <is>
+          <t>The sequencing result depends on the F/I polling default (10s tick, post on 2-of-3 quorum). The model doesn't let the observer use TCP connection identity (5-tuples), which favors the defender at the first hop. Latency ranges and the background traffic mix are Claude Code's defaults, tagged in params.py.</t>
+        </is>
+      </c>
+      <c r="C9" s="32" t="inlineStr">
+        <is>
+          <t>NOTE</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="100" customHeight="1">
+      <c r="A10" s="24" t="inlineStr">
+        <is>
+          <t>Where the full results live</t>
+        </is>
+      </c>
+      <c r="B10" s="7" t="inlineStr">
+        <is>
+          <t>GPAExperiment/level3/ in the repo: RESULTS.md, README.md, results/summary.csv, results/sweep.png. Includes two models beyond the original spec, both marked in the README: a literal reference simulator (real crypto, tick-by-tick lottery) used to validate the fast vectorized sweep engine, and the two ground-truth bound models. Full sweep runtime: ~55 minutes on 4 cores, resumable.</t>
+        </is>
+      </c>
+      <c r="C10" s="32" t="inlineStr">
+        <is>
+          <t>NOTE</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Adopt F/I registry hold as default; keep CV-1/2 hold as rejected comparison
F and I each hold their registry posting in the lottery on their own,
independent node clocks (Level 3!B6, B13). The CV-1/2 hold and the
original no-hold protocol are pinned as labelled comparisons. Adds the
hold to the reference simulator, a fresh-phase-per-posting check variant,
a test that F/I hold clocks are independent, and the updated workbook.
Results for the adopted configuration follow in a separate commit.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TXJ7s8Q6PbdYqCeuNUfpZe
</commit_message>
<xml_diff>
--- a/GPAExperiment/Birthmark_Traffic_Analysis_Catalog.xlsx
+++ b/GPAExperiment/Birthmark_Traffic_Analysis_Catalog.xlsx
@@ -2027,7 +2027,7 @@
       <c r="J26" s="5" t="n"/>
       <c r="K26" s="5" t="inlineStr">
         <is>
-          <t>The submission-to-entry-node step is internal to one Registry node (F/I is co-located with a blockchain node there), not a network event. Only the subsequent gossip fan-out is externally observable. Substrate's transport (libp2p + Noise) encrypts gossip content hop-to-hop by default, so the signature isn't plaintext to an outside GPA — though every node along the gossip path sees it decrypted, a different threat than this experiment's. Size and timing metadata aren't covered by that encryption and remain in scope. Stem/fluff gossip restructuring is the intended direction for protecting which node originated a submission, deferred to a later version.</t>
+          <t>The submission-to-entry-node step is internal to one Registry node (F/I is co-located with a blockchain node there), not a network event. Only the subsequent gossip fan-out is externally observable. Substrate's transport (libp2p + Noise) encrypts gossip content hop-to-hop by default, so the signature isn't plaintext to an outside GPA — though every node along the gossip path sees it decrypted, a different threat than this experiment's. Size and timing metadata aren't covered by that encryption and remain in scope. Stem/fluff gossip restructuring is the intended direction for protecting which node originated a submission, deferred to a later version. ADOPTED (Level 3 experiment result): F/I hold before posting, using the same lottery mechanism already specified elsewhere (10s ticks, 8.33% release probability, 5-min cap), rather than posting immediately on detecting 2-of-3 quorum. Measured to narrow the quorum→registry sequencing signal by 35–43% across the sweep. A hold was also tested at CV-1/2 and found to make the signal worse (22–35% stronger) — rejected, not adopted; CV-1/2 has no hold.</t>
         </is>
       </c>
     </row>
@@ -2080,7 +2080,7 @@
       <c r="J27" s="5" t="n"/>
       <c r="K27" s="5" t="inlineStr">
         <is>
-          <t>The submission-to-entry-node step is internal to one Registry node (F/I is co-located with a blockchain node there), not a network event. Only the subsequent gossip fan-out is externally observable. Substrate's transport (libp2p + Noise) encrypts gossip content hop-to-hop by default, so the signature isn't plaintext to an outside GPA — though every node along the gossip path sees it decrypted, a different threat than this experiment's. Size and timing metadata aren't covered by that encryption and remain in scope. Stem/fluff gossip restructuring is the intended direction for protecting which node originated a submission, deferred to a later version.</t>
+          <t>The submission-to-entry-node step is internal to one Registry node (F/I is co-located with a blockchain node there), not a network event. Only the subsequent gossip fan-out is externally observable. Substrate's transport (libp2p + Noise) encrypts gossip content hop-to-hop by default, so the signature isn't plaintext to an outside GPA — though every node along the gossip path sees it decrypted, a different threat than this experiment's. Size and timing metadata aren't covered by that encryption and remain in scope. Stem/fluff gossip restructuring is the intended direction for protecting which node originated a submission, deferred to a later version. ADOPTED (Level 3 experiment result): F/I hold before posting, using the same lottery mechanism already specified elsewhere (10s ticks, 8.33% release probability, 5-min cap), rather than posting immediately on detecting 2-of-3 quorum. Measured to narrow the quorum→registry sequencing signal by 35–43% across the sweep. A hold was also tested at CV-1/2 and found to make the signal worse (22–35% stronger) — rejected, not adopted; CV-1/2 has no hold.</t>
         </is>
       </c>
     </row>
@@ -2904,7 +2904,7 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="220" customHeight="1">
+    <row r="6" ht="240" customHeight="1">
       <c r="A6" s="24" t="inlineStr">
         <is>
           <t>Quorum→registry sequencing</t>
@@ -2912,7 +2912,7 @@
       </c>
       <c r="B6" s="7" t="inlineStr">
         <is>
-          <t>Additional attack, reported alongside the specified one: score GK fan-out timing against Reg-1/Reg-2 gossip timing. Requires a default for when F/I actually post: F/I poll the match boards on the same 10-second tick as the lottery mechanism and post as soon as they observe a 2-of-3 quorum. Experiment result: the sequencing signal traces to C→validator (CV-1/2) having no lottery hold at all — the round trip fires immediately, letting an observer detect credential-chain endings over 99% of the time and giving the sequencing attack its (sub-1/L but real, ~4–6x above true chance) signal. A lottery hold at CV-1/2, or at F/I before posting to the registry, is the concrete next hardening step to close even this weak residual signal — not required by the current result, since it stays under threshold, but a clean fix given the source is now identified.</t>
+          <t>Additional attack, reported alongside the specified one: score GK fan-out timing against Reg-1/Reg-2 gossip timing. ADOPTED CONFIGURATION: F/I hold before posting using the same lottery mechanism specified elsewhere (10s ticks, 8.33% release probability, 5-min cap), rather than posting immediately on detecting 2-of-3 quorum — measured to narrow the sequencing signal 35–43% across the sweep. A hold at CV-1/2 was also tested and is explicitly REJECTED: it makes the signal WORSE (22–35% stronger at every setting), since delaying the credential side makes content more likely to already be waiting at F/I when quorum forms, tightening rather than loosening the timing link. CV-1/2 has no hold. Even with the F/I hold adopted, the signal is narrowed, not eliminated: it remains real but weak (~above true chance, still under 1/L) and uncalibrated (never confident) — not operationally usable by an attacker, but not zero.</t>
         </is>
       </c>
       <c r="C6" s="7" t="inlineStr">
@@ -3001,7 +3001,7 @@
         </is>
       </c>
     </row>
-    <row r="12" ht="150" customHeight="1">
+    <row r="12" ht="170" customHeight="1">
       <c r="A12" s="7" t="inlineStr">
         <is>
           <t>Registry intake and gossip</t>
@@ -3009,7 +3009,7 @@
       </c>
       <c r="B12" s="7" t="inlineStr">
         <is>
-          <t>F/I is co-located with a blockchain node in the same Registry node, so the submission-to-entry-node step is internal, not network-observable; only the subsequent gossip fan-out is external. Substrate's transport (libp2p + Noise) encrypts gossip content hop-to-hop by default, so signatures aren't plaintext to an outside GPA — though every node along the gossip path sees them decrypted. Size and timing metadata aren't covered by that encryption and remain in scope.</t>
+          <t>F/I is co-located with a blockchain node in the same Registry node, so the submission-to-entry-node step is internal, not network-observable; only the subsequent gossip fan-out is external. Substrate's transport (libp2p + Noise) encrypts gossip content hop-to-hop by default, so signatures aren't plaintext to an outside GPA — though every node along the gossip path sees them decrypted. Size and timing metadata aren't covered by that encryption and remain in scope. F/I now hold before posting (same lottery mechanism, 10s ticks/8.33%/5-min cap) rather than posting immediately on quorum detection — see row 6 for why.</t>
         </is>
       </c>
       <c r="C12" s="7" t="inlineStr">
@@ -3018,7 +3018,7 @@
         </is>
       </c>
     </row>
-    <row r="13" ht="220" customHeight="1">
+    <row r="13" ht="260" customHeight="1">
       <c r="A13" s="24" t="inlineStr">
         <is>
           <t>Tech stack</t>
@@ -3026,7 +3026,7 @@
       </c>
       <c r="B13" s="7" t="inlineStr">
         <is>
-          <t>Python. scipy.optimize.linear_sum_assignment provides the Hungarian algorithm for bipartite matching; ssl gives genuine TLS. Lottery timing, CLARIFIED to close an ambiguity Claude Code correctly flagged: "each held packet as a task rolling its release probability each tick" reads naturally as an independent per-packet timer, which is the LEAKY version — confirmed by experiment, it lets an observer pair packets by shared sub-tick phase, defeating both the relay-hop and device-side clock defenses at once. The correct implementation is one shared clock per role, not per packet: one shared, randomly-phased clock per relay node (every packet held at that node rolls on the same ticks, erasing individual arrival phase), and one independently, freshly-drawn phase per channel at the device (so the device's three simultaneous first-hop departures don't share a phase either). Implement the shared clock as its own recurring task that wakes each held packet's check, rather than giving each packet its own independent timer.</t>
+          <t>Python. scipy.optimize.linear_sum_assignment provides the Hungarian algorithm for bipartite matching; ssl gives genuine TLS. Lottery timing, CLARIFIED to close an ambiguity Claude Code correctly flagged: "each held packet as a task rolling its release probability each tick" reads naturally as an independent per-packet timer, which is the LEAKY version — confirmed by experiment, it lets an observer pair packets by shared sub-tick phase, defeating both the relay-hop and device-side clock defenses at once. The correct implementation is one shared clock per role, not per packet: one shared, randomly-phased clock per relay node (every packet held at that node rolls on the same ticks, erasing individual arrival phase), and one independently, freshly-drawn phase per channel at the device (so the device's three simultaneous first-hop departures don't share a phase either). Implement the shared clock as its own recurring task that wakes each held packet's check, rather than giving each packet its own independent timer. Same principle extends to a third role: F and I each hold before posting to the registry (adopted per row 6), and each gets its own independently, freshly-phased clock -- F's hold clock and I's hold clock are not shared or coupled with each other, matching the per-node pattern above. This is the third instance of the same class of leak this project has hit twice already; stated explicitly rather than left to be inferred a third time.</t>
         </is>
       </c>
     </row>
@@ -3321,7 +3321,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="100" customHeight="1">
+    <row r="5" ht="170" customHeight="1">
       <c r="A5" s="24" t="inlineStr">
         <is>
           <t>Sequencing attack (validator reply → registry posts)</t>
@@ -3329,7 +3329,7 @@
       </c>
       <c r="B5" s="7" t="inlineStr">
         <is>
-          <t>Stays under 1/L (~0.58/L), but true chance for this specific attack is ~5x lower than 1/L (the real pairing window is wider than the 2 minutes L is calibrated against), so this is a real, ~4–6x-above-chance signal, not zero signal. Calibration saves it: no prediction was ever confident, and top-decile accuracy is barely above overall accuracy — an attacker can't act on a signal it can't distinguish from noise. Traced to CV-1/2 (C→validator) having no lottery hold at all; see Level 3 Experiment Design, row 6, for the concrete fix.</t>
+          <t>Numbers below reflect the ADOPTED configuration: F/I hold before posting (same lottery mechanism specified elsewhere); CV-1/2 has no hold (tested and rejected — a hold there makes the signal worse, 22–35% stronger, since it removes noise the attack was depending on rather than adding any). With the F/I hold: signal narrowed 35–43% from the as-built baseline, still under 1/L (~0.58/L, though true chance for this attack is ~5x lower than 1/L — so a real, weak signal remains, ~4–6x above true chance). Calibration is what actually neutralizes it: no prediction is ever confident, and top-decile accuracy is barely above overall accuracy — an attacker can't act on a signal it can't distinguish from noise. See Level 3 Experiment Design, row 6, for the full finding.</t>
         </is>
       </c>
       <c r="C5" s="31" t="inlineStr">
@@ -3389,7 +3389,7 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="100" customHeight="1">
+    <row r="9" ht="130" customHeight="1">
       <c r="A9" s="24" t="inlineStr">
         <is>
           <t>Assumptions the results rest on</t>
@@ -3397,7 +3397,7 @@
       </c>
       <c r="B9" s="7" t="inlineStr">
         <is>
-          <t>The sequencing result depends on the F/I polling default (10s tick, post on 2-of-3 quorum). The model doesn't let the observer use TCP connection identity (5-tuples), which favors the defender at the first hop. Latency ranges and the background traffic mix are Claude Code's defaults, tagged in params.py.</t>
+          <t>The sequencing result depends on the F/I polling default (10s tick, detect 2-of-3 quorum) plus the adopted post-detection hold (same lottery mechanism, each of F and I on its own independent clock). The model doesn't let the observer use TCP connection identity (5-tuples), which favors the defender at the first hop. Latency ranges and the background traffic mix (25 clients/node, 90% casual) are Claude Code's defaults, tagged in params.py — a sensitivity check across 0–100 clients/node left every conclusion unchanged, so the headline result isn't fragile to this particular modeling choice.</t>
         </is>
       </c>
       <c r="C9" s="32" t="inlineStr">

</xml_diff>